<commit_message>
R1ter - output matches latest draft - minor issues left: readme title, requirements, python libraries
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/econ0763/Downloads/JPE/JPE-Jeenas-20240482/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29C3ABE-6B40-2947-8941-A6DB4DA93F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A4EF06-592D-2F47-B06E-7E9895827F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="26860" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="175">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -550,72 +550,6 @@
   </si>
   <si>
     <t>code/Julia/Julia_model_code/auxiliary_model_functions.jl:534</t>
-  </si>
-  <si>
-    <t>No, different</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Linked generated Section 4.2 numbers differ from paper: saved 0.52-&gt;0.23 and 0.41-&gt;0.36; paper reports 0.53-&gt;0.24 and 0.43-&gt;0.39.</t>
-  </si>
-  <si>
-    <t>Saved Table 2 model values differ from paper: pre model 13.65, -0.053, 0.769 vs paper 14.73, -0.049, 0.793; post -0.060, 0.931 vs paper -0.059, 0.953.</t>
-  </si>
-  <si>
-    <t>Model calibration components differ: saved freq(D=1)=0.255 and E[n0]/E[n]=0.26; paper reports 0.252 and 0.25.</t>
-  </si>
-  <si>
-    <t>Model column differs in several untargeted moments, e.g. saved -0.231, 0.122, 0.046, 0.054, 0.017, 0.236, 0.273 vs paper -0.228, 0.125, 0.049, 0.061, 0.014, 0.221, 0.283.</t>
-  </si>
-  <si>
-    <t>Saved model regression table differs from paper in coefficients and observations, e.g. leverage first row 0.364/0.184/0.310 vs paper 0.351/0.169/0.292.</t>
-  </si>
-  <si>
-    <t>Saved model R2 table differs from paper, e.g. leverage 0.73/0.08/0.53 vs paper 0.70/0.07/0.49; liquidity 0.80/0.71/0.57 vs paper 0.95/0.80/0.69.</t>
-  </si>
-  <si>
-    <t>Table component differs slightly: saved liquidity public-private difference 0.047; paper reports 0.048.</t>
-  </si>
-  <si>
-    <t>Linked isolated liquid-asset-return-shock text differs: saved -0.43% pre and -0.57% post; paper reports -0.47% and -0.60%.</t>
-  </si>
-  <si>
-    <t>Linked Appendix B.11.2 decomposition text differs: saved Q share about 3/5 and rb+rm about 2/5; paper reports Q about 2/5 and rb+rm about 3/5.</t>
-  </si>
-  <si>
-    <t>Model line below the one in paper</t>
-  </si>
-  <si>
-    <t>Panel b differs</t>
-  </si>
-  <si>
-    <t>Post-90 differs; Linked Section 5.2 auxiliary numbers differ: saved rm/rb peak ratio 0.26 pre and 0.47 post, GE-PE Q share 1.05; paper reports about 1/3 to 1/2 and about 2/3 Q share.</t>
-  </si>
-  <si>
-    <t>Panel a differs slightly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Differs slightly </t>
-  </si>
-  <si>
-    <t>Replicated 0.52-&gt;0.23 and 0.41-&gt;0.36; paper reports 0.53-&gt;0.24 and 0.43-&gt;0.39.</t>
-  </si>
-  <si>
-    <t>Replicated aggregate debt-to-capital changes by -0.002, roughly -0.2pp; paper says only 0.1pp.</t>
-  </si>
-  <si>
-    <t>Replicated rm/rb peak ratio 0.26 pre and 0.47 post vs about 1/3 to 1/2 in paper; GE-PE Q share 1.05 vs about 2/3 in paper; isolated rm shock -0.43/-0.57 vs -0.47/-0.60.</t>
-  </si>
-  <si>
-    <t>Replicated footnote value is 4.5% of net worth; paper footnote reports about 4.4%.</t>
-  </si>
-  <si>
-    <t>Replicated mean b/k 0.294 and BA-BN 0.281, elasticities 0.144/-0.134; paper reports about 0.31, 0.296, and 0.204/-0.113.</t>
-  </si>
-  <si>
-    <t>Replicated Q share about 3/5 and rb+rm about 2/5; paper reports Q about 2/5 and rb+rm about 3/5.</t>
   </si>
 </sst>
 </file>
@@ -1257,9 +1191,6 @@
       <c r="D20" t="s">
         <v>41</v>
       </c>
-      <c r="E20" t="s">
-        <v>176</v>
-      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
@@ -1313,11 +1244,8 @@
       <c r="C24" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D24" t="s">
-        <v>175</v>
-      </c>
-      <c r="E24" t="s">
-        <v>177</v>
+      <c r="D24" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1344,12 +1272,10 @@
       <c r="C26" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D26" t="s">
-        <v>175</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>186</v>
-      </c>
+      <c r="D26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
@@ -1361,12 +1287,10 @@
       <c r="C27" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D27" t="s">
-        <v>175</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>187</v>
-      </c>
+      <c r="D27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="2"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
@@ -1378,11 +1302,8 @@
       <c r="C28" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D28" t="s">
-        <v>175</v>
-      </c>
-      <c r="E28" t="s">
-        <v>188</v>
+      <c r="D28" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1409,11 +1330,8 @@
       <c r="C30" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D30" t="s">
-        <v>175</v>
-      </c>
-      <c r="E30" t="s">
-        <v>178</v>
+      <c r="D30" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1706,11 +1624,8 @@
       <c r="C51" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D51" t="s">
-        <v>175</v>
-      </c>
-      <c r="E51" t="s">
-        <v>179</v>
+      <c r="D51" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1723,11 +1638,8 @@
       <c r="C52" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D52" t="s">
-        <v>175</v>
-      </c>
-      <c r="E52" t="s">
-        <v>180</v>
+      <c r="D52" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1740,11 +1652,8 @@
       <c r="C53" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D53" t="s">
-        <v>175</v>
-      </c>
-      <c r="E53" t="s">
-        <v>181</v>
+      <c r="D53" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1757,11 +1666,8 @@
       <c r="C54" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D54" t="s">
-        <v>175</v>
-      </c>
-      <c r="E54" t="s">
-        <v>182</v>
+      <c r="D54" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1774,11 +1680,8 @@
       <c r="C55" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D55" t="s">
-        <v>175</v>
-      </c>
-      <c r="E55" t="s">
-        <v>183</v>
+      <c r="D55" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -1820,11 +1723,9 @@
         <v>120</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>189</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="E58" s="2"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
@@ -1836,12 +1737,10 @@
       <c r="C59" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D59" t="s">
-        <v>175</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="D59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E59" s="2"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
@@ -1853,12 +1752,10 @@
       <c r="C60" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D60" t="s">
-        <v>175</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>190</v>
-      </c>
+      <c r="D60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E60" s="2"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
@@ -1912,11 +1809,8 @@
       <c r="C64" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D64" t="s">
-        <v>175</v>
-      </c>
-      <c r="E64" t="s">
-        <v>184</v>
+      <c r="D64" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
@@ -1972,11 +1866,9 @@
         <v>140</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>190</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="E68" s="2"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
@@ -1988,11 +1880,8 @@
       <c r="C69" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D69" t="s">
-        <v>175</v>
-      </c>
-      <c r="E69" t="s">
-        <v>185</v>
+      <c r="D69" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -2014,9 +1903,6 @@
       <c r="D71" t="s">
         <v>41</v>
       </c>
-      <c r="E71" t="s">
-        <v>176</v>
-      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
@@ -2070,11 +1956,8 @@
       <c r="C75" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D75" t="s">
-        <v>175</v>
-      </c>
-      <c r="E75" t="s">
-        <v>191</v>
+      <c r="D75" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -2087,11 +1970,8 @@
       <c r="C76" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="D76" t="s">
-        <v>175</v>
-      </c>
-      <c r="E76" t="s">
-        <v>192</v>
+      <c r="D76" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -2104,11 +1984,8 @@
       <c r="C77" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D77" t="s">
-        <v>175</v>
-      </c>
-      <c r="E77" t="s">
-        <v>193</v>
+      <c r="D77" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -2121,11 +1998,8 @@
       <c r="C78" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D78" t="s">
-        <v>175</v>
-      </c>
-      <c r="E78" t="s">
-        <v>194</v>
+      <c r="D78" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -2156,7 +2030,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>161</v>
       </c>
@@ -2170,7 +2044,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>163</v>
       </c>
@@ -2180,14 +2054,11 @@
       <c r="C82" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="D82" t="s">
-        <v>175</v>
-      </c>
-      <c r="E82" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D82" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>165</v>
       </c>
@@ -2201,7 +2072,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>167</v>
       </c>
@@ -2215,7 +2086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>170</v>
       </c>
@@ -2229,7 +2100,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>172</v>
       </c>
@@ -2239,16 +2110,13 @@
       <c r="C86" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="D86" t="s">
-        <v>175</v>
-      </c>
-      <c r="E86" t="s">
-        <v>196</v>
+      <c r="D86" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D86" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="D1:D54 E30 E51:E54 D55:E55 D56:D1048576 E58 E68">
+  <conditionalFormatting sqref="E30 E51:E55 E58 E68 D1:D1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",D1)))</formula>
     </cfRule>

</xml_diff>